<commit_message>
feat: integrate cfg-luban runtime and drive rank logic from TbRank config
</commit_message>
<xml_diff>
--- a/designer_cfg/Datas/__enums__.xlsx
+++ b/designer_cfg/Datas/__enums__.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace2\luban_examples\MiniTemplate\Datas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\repo\example-proj-cfg\designer_cfg\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57E1AAA0-A88D-4E41-AC05-256E9DB382D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A49FD42F-7CE2-426B-843D-86E9D0C799D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8060" yWindow="5510" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="28">
   <si>
     <t>##var</t>
   </si>
@@ -77,13 +77,49 @@
   </si>
   <si>
     <t>注释</t>
+  </si>
+  <si>
+    <t>RankType</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>市排行榜</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>省排行榜</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>小区榜</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>全区榜</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>City</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Province</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Zone</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AllZone</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -94,6 +130,14 @@
     <font>
       <sz val="9"/>
       <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -141,7 +185,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -150,6 +194,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -429,21 +479,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:L7"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="20.875" customWidth="1"/>
-    <col min="4" max="5" width="14.125" customWidth="1"/>
-    <col min="6" max="6" width="9.375" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="5" width="14.08203125" customWidth="1"/>
+    <col min="6" max="6" width="9.33203125" customWidth="1"/>
     <col min="7" max="7" width="5" customWidth="1"/>
     <col min="8" max="8" width="13.5" customWidth="1"/>
-    <col min="9" max="9" width="5.25" customWidth="1"/>
-    <col min="10" max="10" width="12.125" customWidth="1"/>
-    <col min="11" max="11" width="15.125" customWidth="1"/>
+    <col min="9" max="9" width="11.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.08203125" customWidth="1"/>
+    <col min="11" max="11" width="15.08203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -465,15 +515,15 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
+      <c r="L1" s="5"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -499,7 +549,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="99" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" ht="99" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -528,6 +578,59 @@
         <v>18</v>
       </c>
       <c r="L3" s="1"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" t="b">
+        <v>0</v>
+      </c>
+      <c r="D4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H5" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="J5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J7">
+        <v>4</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>